<commit_message>
Combine comparison into one image and add a per-product usage guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DNFWtABRwmefxWQhJgZ3SK
</commit_message>
<xml_diff>
--- a/car-wash/suppliers/مقارنة-الموردين.xlsx
+++ b/car-wash/suppliers/مقارنة-الموردين.xlsx
@@ -13,7 +13,7 @@
     <sheet name="سلة الشراء المقترحة" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">المقارنة!$A$1:$K$43</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">المقارنة!$A$1:$K$44</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="160">
   <si>
     <t xml:space="preserve">المادة</t>
   </si>
@@ -138,51 +138,60 @@
     <t xml:space="preserve">2. واكس سبراي</t>
   </si>
   <si>
+    <t xml:space="preserve">Last Touch Express</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رش ومسح بدون ماي — متوفر 4.5 لتر (اسألهم)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceramic Spray Coating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رش ومسح — بديل جملة (بدون بخاخ)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Profiline Spray &amp; Seal</t>
   </si>
   <si>
+    <t xml:space="preserve">✗ يحتاج شطف بالماي — ما يناسبكم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xtreme Spray &amp; Seal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quik Wax 24oz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">السعر غير مؤكد (4.5 أو 4.99)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ProTech Kuwait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maxi Shine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فرنسا 🇫🇷 (ماركتهم)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">★★★★ (ماركة محل، غالي)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+965 9691 2001 / 2491 0075</t>
+  </si>
+  <si>
+    <t xml:space="preserve">غير متوفر وقت البحث</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. منظف متعدد APC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profiline Multistar</t>
+  </si>
+  <si>
     <t xml:space="preserve">حجم جملة</t>
   </si>
   <si>
-    <t xml:space="preserve">Xtreme Spray &amp; Seal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Touch Express</t>
-  </si>
-  <si>
-    <t xml:space="preserve">الحجم مو مذكور (غالبًا 500 مل)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quik Wax 24oz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">السعر غير مؤكد (4.5 أو 4.99)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ProTech Kuwait</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maxi Shine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">فرنسا 🇫🇷 (ماركتهم)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">★★★★ (ماركة محل، غالي)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+965 9691 2001 / 2491 0075</t>
-  </si>
-  <si>
-    <t xml:space="preserve">غير متوفر وقت البحث</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. منظف متعدد APC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profiline Multistar</t>
-  </si>
-  <si>
     <t xml:space="preserve">Profiline MultiClean Alkaline</t>
   </si>
   <si>
@@ -441,7 +450,7 @@
     <t xml:space="preserve">واكس سبراي</t>
   </si>
   <si>
-    <t xml:space="preserve">Sonax Profiline Spray &amp; Seal 5L</t>
+    <t xml:space="preserve">MA-FRA Last Touch Express 500ml</t>
   </si>
   <si>
     <t xml:space="preserve">منظف متعدد</t>
@@ -1118,7 +1127,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="26"/>
@@ -1300,34 +1309,34 @@
       </c>
       <c r="K5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5000</v>
+        <v>500</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>16.3</v>
+        <v>3</v>
       </c>
       <c r="G6" s="3" t="n">
         <f aca="false">F6/E6*100</f>
-        <v>0.326</v>
+        <v>0.6</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>38</v>
@@ -1350,14 +1359,14 @@
         <v>14</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>750</v>
+        <v>5000</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.1</v>
+        <v>18.8</v>
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">F7/E7*100</f>
-        <v>0.413333333333333</v>
+        <v>0.376</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>15</v>
@@ -1365,73 +1374,76 @@
       <c r="I7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="6"/>
+      <c r="J7" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>36</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>27</v>
+        <v>14</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>5000</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>28</v>
+        <v>16.3</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <f aca="false">F8/E8*100</f>
+        <v>0.326</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
         <v>36</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>710</v>
+        <v>750</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4.99</v>
+        <v>3.1</v>
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">F9/E9*100</f>
-        <v>0.702816901408451</v>
+        <v>0.413333333333333</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K9" s="6"/>
     </row>
@@ -1440,124 +1452,126 @@
         <v>36</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="D10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>710</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <f aca="false">F10/E10*100</f>
+        <v>0.702816901408451</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="C11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J10" s="6" t="s">
+      <c r="H11" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="K10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="I11" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="J11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="C12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E12" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F12" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G11" s="3" t="n">
-        <f aca="false">F11/E11*100</f>
+      <c r="G12" s="3" t="n">
+        <f aca="false">F12/E12*100</f>
         <v>0.25</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K11" s="2" t="s">
+      <c r="J12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <f aca="false">F12/E12*100</f>
-        <v>0.45</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>14</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>13</v>
+        <v>4.5</v>
       </c>
       <c r="G13" s="5" t="n">
         <f aca="false">F13/E13*100</f>
-        <v>0.26</v>
+        <v>0.45</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>15</v>
@@ -1565,38 +1579,37 @@
       <c r="I13" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="4" t="s">
-        <v>38</v>
-      </c>
+      <c r="J13" s="4"/>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>27</v>
+        <v>14</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>5000</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>28</v>
+        <v>13</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <f aca="false">F14/E14*100</f>
+        <v>0.26</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="J14" s="4" t="s">
         <v>54</v>
@@ -1605,126 +1618,125 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>27</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>4.95</v>
+        <v>2.5</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>58</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>27</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>1.5</v>
+        <v>4.95</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H16" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="K16" s="4"/>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="E17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="I17" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <f aca="false">F17/E17*100</f>
-        <v>0.43</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="K17" s="6"/>
+      <c r="J17" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>6.3</v>
+        <v>21.5</v>
       </c>
       <c r="G18" s="7" t="n">
         <f aca="false">F18/E18*100</f>
-        <v>0.63</v>
+        <v>0.43</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>15</v>
@@ -1732,356 +1744,358 @@
       <c r="I18" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J18" s="6"/>
+      <c r="J18" s="6" t="s">
+        <v>54</v>
+      </c>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B19" s="2" t="s">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <f aca="false">F19/E19*100</f>
+        <v>0.63</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F19" s="3" t="n">
+      <c r="F20" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I20" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="K19" s="2" t="s">
+      <c r="J20" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K20" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>27</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>2</v>
+        <v>4.75</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>28</v>
       </c>
       <c r="H21" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="K21" s="6"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E22" s="4" t="s">
+      <c r="D22" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K22" s="6"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23" s="5" t="n">
         <v>1.5</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G23" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H22" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="K22" s="4"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="2" t="s">
+      <c r="H23" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="K23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B24" s="4" t="s">
+      <c r="B25" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="C25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E25" s="4" t="n">
         <v>400</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F25" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <f aca="false">F24/E24*100</f>
-        <v>1</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>473</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>4.99</v>
       </c>
       <c r="G25" s="5" t="n">
         <f aca="false">F25/E25*100</f>
-        <v>1.05496828752643</v>
+        <v>1</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>473</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>28</v>
+        <v>4.99</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <f aca="false">F26/E26*100</f>
+        <v>1.05496828752643</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="2" t="s">
+      <c r="A27" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" s="2" t="s">
+      <c r="C28" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F28" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="I28" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2" t="s">
+      <c r="J28" s="2"/>
+      <c r="K28" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E28" s="6" t="n">
-        <v>750</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <f aca="false">F28/E28*100</f>
-        <v>0.333333333333333</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I28" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G29" s="7" t="n">
         <f aca="false">F29/E29*100</f>
-        <v>0.3</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>15</v>
@@ -2092,466 +2106,498 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>27</v>
+        <v>14</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>1000</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>28</v>
+        <v>3</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <f aca="false">F30/E30*100</f>
+        <v>0.3</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>710</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>22</v>
+        <v>48</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>4.4</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>28</v>
       </c>
       <c r="H31" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>710</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I31" s="6" t="s">
+      <c r="I32" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="J31" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="K31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B32" s="2" t="s">
+      <c r="J32" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="K32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="C33" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E33" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="F33" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="I33" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2" t="s">
+      <c r="J33" s="2"/>
+      <c r="K33" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B33" s="4" t="s">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C33" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" s="4" t="s">
+      <c r="C34" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E34" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="F33" s="5" t="n">
+      <c r="F34" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="G33" s="5" t="n">
-        <f aca="false">F33/E33*100</f>
+      <c r="G34" s="5" t="n">
+        <f aca="false">F34/E34*100</f>
         <v>1.8</v>
       </c>
-      <c r="H33" s="4" t="s">
+      <c r="H34" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I33" s="4" t="s">
+      <c r="I34" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J33" s="4" t="s">
+      <c r="J34" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="K34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="K33" s="4"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D34" s="4" t="s">
+      <c r="B35" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="C35" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F34" s="5" t="n">
+      <c r="F35" s="5" t="n">
         <v>2.75</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G35" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H34" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="J34" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="K34" s="4"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+      <c r="H35" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="K35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <f aca="false">F37/E37*100</f>
+        <v>1.8</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J37" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E35" s="2" t="s">
+      <c r="K37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F35" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="G35" s="2" t="s">
+      <c r="F38" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H35" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2" t="s">
+      <c r="H38" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="K38" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B36" s="6" t="s">
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D36" s="6" t="s">
+      <c r="C39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D39" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F36" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="G36" s="7" t="n">
-        <f aca="false">F36/E36*100</f>
-        <v>1.8</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I36" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J36" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="K36" s="6"/>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F37" s="3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I38" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J38" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="K38" s="4"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>27</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="G39" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J39" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>99</v>
+      </c>
       <c r="K39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>27</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>3.85</v>
+        <v>2</v>
       </c>
       <c r="G40" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E41" s="2" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F41" s="3" t="n">
+      <c r="F41" s="5" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+    </row>
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F42" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="G42" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H41" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="K41" s="2" t="s">
+      <c r="H42" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K42" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B42" s="6" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B43" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C42" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="D42" s="6" t="s">
+      <c r="C43" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F42" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I42" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6"/>
-    </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>14</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>27</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>1.55</v>
+        <v>1</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>28</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F44" s="7" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K43"/>
+  <autoFilter ref="A1:K44"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2583,22 +2629,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2606,7 +2652,7 @@
         <v>24</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>26</v>
@@ -2615,13 +2661,13 @@
         <v>30</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2629,7 +2675,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>14</v>
@@ -2638,56 +2684,56 @@
         <v>16</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>28</v>
@@ -2698,7 +2744,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>20</v>
@@ -2707,10 +2753,10 @@
         <v>22</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>28</v>
@@ -2721,7 +2767,7 @@
         <v>32</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>14</v>
@@ -2730,13 +2776,13 @@
         <v>34</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2770,30 +2816,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D2" s="11" t="n">
         <v>1</v>
@@ -2808,34 +2854,34 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>16.3</v>
+        <v>3</v>
       </c>
       <c r="F3" s="12" t="n">
         <f aca="false">D3*E3</f>
-        <v>16.3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>139</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>136</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>1</v>
@@ -2850,13 +2896,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>2</v>
@@ -2871,13 +2917,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>2</v>
@@ -2892,13 +2938,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>2</v>
@@ -2913,13 +2959,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>1</v>
@@ -2934,13 +2980,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>1</v>
@@ -2955,13 +3001,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D10" s="11" t="n">
         <v>20</v>
@@ -2976,13 +3022,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>4</v>
@@ -3001,16 +3047,16 @@
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
       <c r="E12" s="13" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F12" s="13" t="n">
         <f aca="false">SUM(F2:F11)</f>
-        <v>93.3</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>